<commit_message>
Changes 2nd after DB referesh Nov 1 2023
</commit_message>
<xml_diff>
--- a/TestData/TMTI0046461_VerifyCompaniesRelatedListOpportunitiesEngagementEnhancedWithFiltering.xlsx
+++ b/TestData/TMTI0046461_VerifyCompaniesRelatedListOpportunitiesEngagementEnhancedWithFiltering.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64B3390-0B55-44AC-8E87-1ACBE0CDD319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7252E1F-F1D2-4A77-9951-6C46E7F71AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14640" xr2:uid="{D381DC3E-0C7A-48CF-8E3B-36CB765DCADA}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" activeTab="4" xr2:uid="{D381DC3E-0C7A-48CF-8E3B-36CB765DCADA}"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
   <si>
     <t>StdUser</t>
   </si>
@@ -123,19 +123,25 @@
     <t>Burke Williams, Inc.</t>
   </si>
   <si>
-    <t>Project Chavez</t>
-  </si>
-  <si>
     <t>Project Miura</t>
   </si>
   <si>
     <t>120228</t>
   </si>
   <si>
-    <t>120227</t>
-  </si>
-  <si>
-    <t>Book Prep/Underwriting</t>
+    <t>Burke Williams Opp</t>
+  </si>
+  <si>
+    <t>125589</t>
+  </si>
+  <si>
+    <t>Burke Williams Eng</t>
+  </si>
+  <si>
+    <t>125590</t>
+  </si>
+  <si>
+    <t>Advisory</t>
   </si>
 </sst>
 </file>
@@ -159,12 +165,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -179,12 +191,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,20 +512,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7DDA40C-CB43-498D-A2ED-A0851564593B}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -537,8 +550,14 @@
       <c r="H1" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -563,8 +582,14 @@
       <c r="H2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -572,23 +597,26 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
         <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>31</v>
-      </c>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -671,8 +699,8 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>